<commit_message>
checklist and test-case have been changed
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="60">
   <si>
     <t>ID</t>
   </si>
@@ -196,6 +196,9 @@
   </si>
   <si>
     <t>CH-025</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
 </sst>
 </file>
@@ -220,6 +223,7 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <i/>
       <sz val="11"/>
       <color theme="1"/>
@@ -278,7 +282,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -599,7 +603,9 @@
       <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -611,7 +617,9 @@
       <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -623,7 +631,9 @@
       <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -635,7 +645,9 @@
       <c r="C6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
@@ -655,7 +667,9 @@
       <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="2"/>
+      <c r="D8" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -667,7 +681,9 @@
       <c r="C9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="2"/>
+      <c r="D9" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -679,7 +695,9 @@
       <c r="C10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="2"/>
+      <c r="D10" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -691,7 +709,9 @@
       <c r="C11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -703,7 +723,9 @@
       <c r="C12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="2"/>
+      <c r="D12" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -715,7 +737,9 @@
       <c r="C13" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="2"/>
+      <c r="D13" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
@@ -735,7 +759,9 @@
       <c r="C15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="2"/>
+      <c r="D15" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
@@ -747,7 +773,9 @@
       <c r="C16" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="2"/>
+      <c r="D16" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
@@ -759,7 +787,9 @@
       <c r="C17" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="2"/>
+      <c r="D17" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
@@ -771,7 +801,9 @@
       <c r="C18" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="2"/>
+      <c r="D18" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
@@ -783,7 +815,9 @@
       <c r="C19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="2"/>
+      <c r="D19" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
@@ -795,7 +829,9 @@
       <c r="C20" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="2"/>
+      <c r="D20" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
@@ -815,7 +851,9 @@
       <c r="C22" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="2"/>
+      <c r="D22" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
@@ -827,7 +865,9 @@
       <c r="C23" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="2"/>
+      <c r="D23" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
@@ -839,7 +879,9 @@
       <c r="C24" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D24" s="2"/>
+      <c r="D24" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
@@ -851,7 +893,9 @@
       <c r="C25" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D25" s="2"/>
+      <c r="D25" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
@@ -871,7 +915,9 @@
       <c r="C27" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="2"/>
+      <c r="D27" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
@@ -883,7 +929,9 @@
       <c r="C28" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D28" s="2"/>
+      <c r="D28" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
@@ -895,7 +943,9 @@
       <c r="C29" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D29" s="2"/>
+      <c r="D29" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
@@ -907,7 +957,9 @@
       <c r="C30" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D30" s="2"/>
+      <c r="D30" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
@@ -919,7 +971,9 @@
       <c r="C31" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="2"/>
+      <c r="D31" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>